<commit_message>
feat: Initialize frontend with React and Vite, add main entry point
feat: Implement Annotate page for asset annotation with configuration and automation features

feat: Create Extract page for extracting assets from the floorplan with verification and export options

build: Configure Vite for development with proxy settings for API calls

chore: Add start-dev.bat script for launching Flask API and Vite dev server simultaneously

chore: Add .gitkeep to uploads directory to ensure it is tracked in version control
</commit_message>
<xml_diff>
--- a/ids.xlsx
+++ b/ids.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Development\App\Asset-Annotation-Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{758AC756-B5C8-4F04-98A6-0ABBA3DDD34B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C101756-0DAB-4B21-B38E-88252C7092C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23040" yWindow="156" windowWidth="21600" windowHeight="11292" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -369,9 +369,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="28.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -382,40 +385,41 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1010001</v>
+        <v>70101</v>
       </c>
       <c r="B2">
-        <v>100</v>
+        <v>147.26840625</v>
       </c>
       <c r="C2">
-        <v>100</v>
+        <v>117.25</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1010002</v>
+        <v>70102</v>
       </c>
       <c r="B3">
-        <v>120</v>
+        <v>147.26840625</v>
       </c>
       <c r="C3">
-        <v>100</v>
+        <v>141.25</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>1010003</v>
+        <v>70103</v>
       </c>
       <c r="B4">
-        <v>140</v>
+        <v>211.27640625000001</v>
       </c>
       <c r="C4">
-        <v>100</v>
+        <v>131.25</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>